<commit_message>
hardware: generator ladder all 10k, R as parallel pairs, filter corner now 33 kHz; schematic exports regenerated
</commit_message>
<xml_diff>
--- a/Oscil_bill_of_materials_bom.xlsx
+++ b/Oscil_bill_of_materials_bom.xlsx
@@ -638,7 +638,7 @@
     <row r="3" ht="14.25" customHeight="1" s="30">
       <c r="A3" s="34" t="inlineStr">
         <is>
-          <t>Paul Simbulan · Rev 0.3 · 28-Sep-2026</t>
+          <t>Paul Simbulan · Rev 0.4 · 30-Sep-2026</t>
         </is>
       </c>
       <c r="E3" s="35" t="inlineStr">
@@ -647,7 +647,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="14.25" customHeight="1" s="30">
       <c r="A5" s="36" t="inlineStr">
         <is>
@@ -1022,7 +1021,7 @@
       </c>
       <c r="I13" s="39" t="inlineStr">
         <is>
-          <t>No 20k/75R/51R/150R/750k/249k in kit: 20k = 2x10k in series (ladder, match pairs), 75R = 100R||330R (76.7R), 51R = 47R+4.7R, 150R = 100R+47R, 750k = 680k+68k, 249k = 220k+33k. 10k budget: ladder 25 + tie-offs 4 = 29 of 40</t>
+          <t>No 75R/51R/150R/750k/249k in kit: ladder is all 10k (2R = 10k, R = 2x10k in parallel = 5k, match by meter), 75R = 100R||330R (76.7R), 51R = 47R+4.7R, 150R = 100R+47R, 750k = 680k+68k, 249k = 220k+33k. 10k budget: ladder 23 + tie-offs 4 = 27 of 40</t>
         </is>
       </c>
       <c r="J13" s="41" t="inlineStr">
@@ -1969,7 +1968,6 @@
         </is>
       </c>
     </row>
-    <row r="40"/>
     <row r="41" ht="14.25" customHeight="1" s="30">
       <c r="D41" s="50" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
bom: fix ESP32-S3, FNIRSI and FX2LP links, make kit links clickable
</commit_message>
<xml_diff>
--- a/Oscil_bill_of_materials_bom.xlsx
+++ b/Oscil_bill_of_materials_bom.xlsx
@@ -174,7 +174,7 @@
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -346,6 +346,9 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
     </xf>
   </cellXfs>
   <cellStyles count="7">
@@ -1069,7 +1072,7 @@
           <t>Rev A: 470p, 1n, 2.2n, 10n, 1u from here. Dielectric unstated, DMM-verify. C0G for Rev B</t>
         </is>
       </c>
-      <c r="J14" s="29" t="inlineStr">
+      <c r="J14" s="58" t="inlineStr">
         <is>
           <t>https://a.co/d/0dSCox0r</t>
         </is>
@@ -1273,7 +1276,7 @@
       </c>
       <c r="J20" s="41" t="inlineStr">
         <is>
-          <t>https://a.co/d/0bcMUA3H</t>
+          <t>https://a.co/d/07rz7Fj1</t>
         </is>
       </c>
     </row>
@@ -1879,7 +1882,7 @@
       </c>
       <c r="J37" s="41" t="inlineStr">
         <is>
-          <t>https://a.co/d/01g446Bb</t>
+          <t>https://a.co/d/0hUidHrU</t>
         </is>
       </c>
     </row>
@@ -1924,7 +1927,7 @@
       </c>
       <c r="J38" s="41" t="inlineStr">
         <is>
-          <t>https://a.co/d/01g446Bb</t>
+          <t>https://a.co/d/0aDcLZeU</t>
         </is>
       </c>
     </row>
@@ -2089,16 +2092,20 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J10" display="https://a.co/d/0cBGTOYl" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J11" display="https://a.co/d/0bSwA5N5" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J12" display="https://a.co/d/09HmNMVi" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J16" display="https://www.digikey.com/en/products/detail/microchip-technology/MCP1700-3302E-TO/652680?s=N4IgTCBcDaILIGEAKBGA7ABgwWgMy4zAFEB6AFQHlsA5AEQAIQBdAXyA" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J17" display="https://a.co/d/02AsqIvb" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J20" display="https://a.co/d/0bcMUA3H" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J22" display="https://www.digikey.com/en/products/detail/orient-display/AFY800480B0-7-0N12NTM-C/12089250?s=N4IgTCBcDa4KwBYEFoCCAxAmgDgAy4TwCFdkB2EAXQF8g" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J23" display="https://www.digikey.com/en/products/detail/adafruit-industries-llc/1932/5761222?s=N4IgTCBcDaIAQEYCsYAcBaBAWJX0DkAREAXQF8g" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J24" display="https://a.co/d/07UskTTP" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J27" display="https://a.co/d/0f5mQg6T" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J31" display="https://www.digikey.com/en/products/detail/sullins-connector-solutions/PRPC040SAAN-RC/2775214?s=N4IgTCBcDaIAQGUCMAGJSCiBhAtAFhRwDkAROEAXQF8g" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J32" display="https://a.co/d/04z6zcu7" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J37" display="https://a.co/d/01g446Bb" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J13" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J14" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J16" display="https://www.digikey.com/en/products/detail/microchip-technology/MCP1700-3302E-TO/652680?s=N4IgTCBcDaILIGEAKBGA7ABgwWgMy4zAFEB6AFQHlsA5AEQAIQBdAXyA" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J17" display="https://a.co/d/02AsqIvb" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J20" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J22" display="https://www.digikey.com/en/products/detail/orient-display/AFY800480B0-7-0N12NTM-C/12089250?s=N4IgTCBcDa4KwBYEFoCCAxAmgDgAy4TwCFdkB2EAXQF8g" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J23" display="https://www.digikey.com/en/products/detail/adafruit-industries-llc/1932/5761222?s=N4IgTCBcDaIAQEYCsYAcBaBAWJX0DkAREAXQF8g" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J24" display="https://a.co/d/07UskTTP" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J27" display="https://a.co/d/0f5mQg6T" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J31" display="https://www.digikey.com/en/products/detail/sullins-connector-solutions/PRPC040SAAN-RC/2775214?s=N4IgTCBcDaIAQGUCMAGJSCiBhAtAFhRwDkAROEAXQF8g" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J32" display="https://a.co/d/04z6zcu7" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J34" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J37" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J38" r:id="rId20"/>
   </hyperlinks>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>